<commit_message>
Merge Taimoor audit: 4 new probe tests (61 total), B-D10 c2 demonstrated, proposed workbook + col F, report/VIVA sync
</commit_message>
<xml_diff>
--- a/workbook/Workbook.xlsx
+++ b/workbook/Workbook.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -489,12 +489,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Structural target</t>
+          <t>Structural-coverage target</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Ref</t>
+          <t>Test-file / evidence reference</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>...ArmedButWaitingBeforeExpiry</t>
+          <t>HysteresisStructural.TrueToFalseArmedButWaitingBeforeExpiry</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>...QuiescentFalseShowsNoArm</t>
+          <t>HysteresisStructural.QuiescentFalseShowsNoArm</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>...NoRequestMeansNoTransition</t>
+          <t>HysteresisStructural.NoRequestMeansNoTransition</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>...FalseToTrueArmTakenWhenExpired</t>
+          <t>HysteresisStructural.FalseToTrueArmTakenWhenExpired</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>...FalseToTrueArmedButWaitingBeforeExpiry</t>
+          <t>HysteresisStructural.FalseToTrueArmedButWaitingBeforeExpiry</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>...QuiescentTrueShowsNoArm</t>
+          <t>HysteresisStructural.QuiescentTrueShowsNoArm</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>...NoRequestMeansNoTransitionUpwards</t>
+          <t>HysteresisStructural.NoRequestMeansNoTransitionUpwards</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>...RepeatRequestKeepsOriginalStamp</t>
+          <t>HysteresisStructural.RepeatRequestKeepsOriginalStamp</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>...AsymmetricWindowsIndependent</t>
+          <t>HysteresisStructural.AsymmetricWindowsIndependent</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>...HysteresisTimesSetPerDirection</t>
+          <t>HysteresisStructural.HysteresisTimesSetPerDirection</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>WarningLadderRungs</t>
+          <t>BatteryStructural.WarningLadderRungs</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>WarningExactThresholdTakesHigherRung</t>
+          <t>BatteryStructural.WarningExactThresholdTakesHigherRung</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>LowVoltageForcesUnconnected</t>
+          <t>BatteryStructural.LowVoltageForcesUnconnected</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>WarningHeldUntilInitialized</t>
+          <t>BatteryStructural.WarningHeldUntilInitialized</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>RlsResetGateFiresPreInit</t>
+          <t>BatteryStructural.RlsResetGateFiresPreInit</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>...BlockedWhenUnconnected</t>
+          <t>BatteryStructural.RlsResetGateBlockedWhenUnconnected</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>...OnlyPreInit</t>
+          <t>BatteryStructural.RlsResetGateOnlyPreInit</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>...BlockedWhenResistanceInvalidated</t>
+          <t>BatteryStructural.RlsResetGateBlockedWhenResistanceInvalidated</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>...BlockedWhenNoCells</t>
+          <t>BatteryStructural.RlsResetGateBlockedWhenNoCells</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>SpikeFaultAboveBoundary</t>
+          <t>BatteryStructural.SpikeFaultAboveBoundary</t>
         </is>
       </c>
     </row>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>...ExactlyAtBoundaryIsClean</t>
+          <t>BatteryStructural.SpikeFaultExactlyAtBoundaryIsClean</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>...NeedsCells</t>
+          <t>BatteryStructural.SpikeFaultNeedsCells</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>SocFusesAndDischargesMonotonically</t>
+          <t>BatteryStructural.SocFusesAndDischargesMonotonically</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>DtClampCapsDischargeIncrement</t>
+          <t>BatteryStructural.DtClampCapsDischargeIncrement</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>ScaleClampedToBand</t>
+          <t>BatteryStructural.ScaleClampedToBand</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>...FallsBackOnNonFinite</t>
+          <t>BatteryStructural.ScaleFallsBackOnNonFinite</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>RemainingTimeNeedsCapacity</t>
+          <t>BatteryStructural.RemainingTimeNeedsCapacity</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>...UnarmedUsesAverage</t>
+          <t>BatteryStructural.RemainingTimeUnarmedUsesAverage</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>ArmedMultirotorUpdatesAverage</t>
+          <t>BatteryStructural.ArmedMultirotorUpdatesAverage</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>...StalePhaseHoldsAverage</t>
+          <t>BatteryStructural.ArmedFixedWingWithStalePhaseHoldsAverage</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>TemperatureRelayedToStatus</t>
+          <t>BatteryStructural.TemperatureRelayedToStatus</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>UpdateAndPublishMatchesSource</t>
+          <t>BatteryStructural.UpdateAndPublishMatchesSource</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>...SkipsOnSourceMismatch</t>
+          <t>BatteryStructural.UpdateAndPublishSkipsOnSourceMismatch</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>OutOfRangeIndexClampsToOne</t>
+          <t>BatteryStructural.OutOfRangeIndexClampsToOne</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>UserInternalResistanceUsedInReset</t>
+          <t>BatteryStructural.UserInternalResistanceUsedInReset</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2048,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>...CorrectsCellVoltage</t>
+          <t>BatteryStructural.UserInternalResistanceCorrectsCellVoltage</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>...FreshLevelPhaseUpdatesAverage</t>
+          <t>BatteryStructural.ArmedFixedWingWithFreshLevelPhaseUpdatesAverage</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>...ZeroDtUpdatesAverageWithoutDt</t>
+          <t>BatteryStructural.ArmedFixedWingZeroDtUpdatesAverageWithoutDt</t>
         </is>
       </c>
     </row>
@@ -2174,34 +2174,34 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>...NonLevelPhaseHoldsAverage</t>
+          <t>BatteryStructural.ArmedFixedWingNonLevelPhaseHoldsAverage</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>PST-01</t>
+          <t>BST-30</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>update + updateIntegral</t>
+          <t>ctor index guard</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>integral frozen when flag cleared, then evolves</t>
+          <t>index 0 exercises `index&lt;1` operand</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>P2/I5, sp1, fb0, dt0.1, flag F then T</t>
+          <t>index 0 (99 covers only `&gt;9`)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>2.0 + int 0; then 2.0 + int 0.5</t>
+          <t>id 1</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2211,39 +2211,39 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>P-D1 F→T</t>
+          <t>L61 second disjunct</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>IntegralFrozenWhenUpdateFlagCleared</t>
+          <t>BatteryStructural.ZeroIndexClampsToOne</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>PST-02</t>
+          <t>BST-31</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>output clamp + integral</t>
+          <t>computeRemainingTime</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>high-side saturation clamps output, integral accumulates (no freeze gate in v1.17.0)</t>
+          <t>armed + NaN current holds average</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>I.5/lim10/out±.2, sp2, fb0, dt.5 ×2</t>
+          <t>ARMED rotary, current NaN</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>0 + int.5; then .2 + int 1.0</t>
+          <t>avg 5.0 (reset, update skipped)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2253,39 +2253,39 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>saturation edges</t>
+          <t>B-D10 c2 vs BST-19</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>SaturationHighClampsOutputIntegralNotFrozen</t>
+          <t>BatteryStructural.ArmedNonFiniteCurrentHoldsAverage</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>PST-03</t>
+          <t>BST-32</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>output clamp + integral</t>
+          <t>computeRemainingTime</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>low-side mirror</t>
+          <t>FW second copy skips transition reset</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>sp−2 mirror</t>
+          <t>ARMED FW ×2 pubs, target 7.0</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>0 + int−.5; then −.2 + int −1.0</t>
+          <t>avg holds 5.0</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -2295,39 +2295,39 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>saturation edges</t>
+          <t>L359 aT,bF</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>SaturationLowClampsOutputIntegralNotFrozen</t>
+          <t>BatteryStructural.FixedWingSecondCopySkipsTransitionReset</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>PST-04</t>
+          <t>BST-33</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>integral unwind</t>
+          <t>computeRemainingTime</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>error reversal under saturation unwinds integral</t>
+          <t>unadvertised topic keeps armed false</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>saturated-high, then sp→−2</t>
+          <t>publish, unadvertise, fresh Battery</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>.2 + int 0.5</t>
+          <t>t finite, avg 5.0, unarmed</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2337,39 +2337,39 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>saturation edges</t>
+          <t>robustness (L356-F investigated)</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>SaturationHighThenReversalUnwindsIntegral</t>
+          <t>BatteryStructural.UnadvertisedTopicHoldsArmedFalse</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>PST-05</t>
+          <t>PST-01</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>updateIntegral</t>
+          <t>update + updateIntegral</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>NaN feedback discards integral candidate</t>
+          <t>integral frozen when flag cleared, then evolves</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>P1/I.1, sp1, fb NaN</t>
+          <t>P2/I5, sp1, fb0, dt0.1, flag F then T</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>NaN out + int 0; then 0 + int 0</t>
+          <t>2.0 + int 0; then 2.0 + int 0.5</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2379,39 +2379,39 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>P-D2 F-path</t>
+          <t>P-D1 F→T</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>NonFiniteIntegralCandidateIsDiscarded_NaN</t>
+          <t>PIDStructural.IntegralFrozenWhenUpdateFlagCleared</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>PST-06</t>
+          <t>PST-02</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>updateIntegral + output clamp</t>
+          <t>output clamp + integral</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>−Inf feedback clamps output, integral held</t>
+          <t>high-side saturation clamps output, integral accumulates (no freeze gate in v1.17.0)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>P1/I.1, sp1, fb −Inf</t>
+          <t>I.5/lim10/out±.2, sp2, fb0, dt.5 ×2</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>+10 + int 0; then 0 + int 0</t>
+          <t>0 + int.5; then .2 + int 1.0</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2421,39 +2421,39 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>P-D2 F-path + clamp</t>
+          <t>saturation edges</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>..._NegInfSaturates</t>
+          <t>PIDStructural.SaturationHighClampsOutputIntegralNotFrozen</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>PST-07</t>
+          <t>PST-03</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>output clamp + integral</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>guard all-false (dt 0, last NaN)</t>
+          <t>low-side mirror</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>D4, fb2.0, dt0, fresh</t>
+          <t>sp−2 mirror</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0 + int−.5; then −.2 + int −1.0</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2463,39 +2463,39 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>P-D3 FF</t>
+          <t>saturation edges</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>DerivativeGuardBlocksWhenNoTimeAndNoHistory</t>
+          <t>PIDStructural.SaturationLowClampsOutputIntegralNotFrozen</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>PST-08</t>
+          <t>PST-04</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>integral unwind</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>time ok, no history (dt .5, last NaN)</t>
+          <t>error reversal under saturation unwinds integral</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>D4, fb2.0, dt.5, fresh</t>
+          <t>saturated-high, then sp→−2</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>.2 + int 0.5</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2505,39 +2505,39 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TF</t>
+          <t>saturation edges</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>...TimeOkButNoHistory</t>
+          <t>PIDStructural.SaturationHighThenReversalUnwindsIntegral</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>PST-09</t>
+          <t>PST-05</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>updateIntegral</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>fully active (PLUS sign, L47)</t>
+          <t>NaN feedback discards integral candidate</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>D4, seed 2.0/.5, then 2.5/.5</t>
+          <t>P1/I.1, sp1, fb NaN</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>+4.0</t>
+          <t>NaN out + int 0; then 0 + int 0</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2547,39 +2547,39 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TT</t>
+          <t>P-D2 F-path</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>...ActiveWhenTimeAndHistory</t>
+          <t>PIDStructural.NonFiniteIntegralCandidateIsDiscarded_NaN</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>PST-10</t>
+          <t>PST-06</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>updateDerivative</t>
+          <t>updateIntegral + output clamp</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>history present but dt 0</t>
+          <t>−Inf feedback clamps output, integral held</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>D4, seed 2.0/.5, then 3.0/dt0</t>
+          <t>P1/I.1, sp1, fb −Inf</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>+10 + int 0; then 0 + int 0</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2589,19 +2589,19 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>P-D3 FT</t>
+          <t>P-D2 F-path + clamp</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>...HistoryButNoTime</t>
+          <t>PIDStructural.NonFiniteIntegralCandidateIsDiscarded_NegInfSaturates</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>PST-11</t>
+          <t>PST-07</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2611,12 +2611,12 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>exact dt==EPS boundary (not &gt;)</t>
+          <t>guard all-false (dt 0, last NaN)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>D4, seed 2.0/.5, then 2.5/dt=EPS</t>
+          <t>D4, fb2.0, dt0, fresh</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2631,19 +2631,19 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>P-D3 boundary</t>
+          <t>P-D3 FF</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>...ExactEpsilonIsNotEnoughTime</t>
+          <t>PIDStructural.DerivativeGuardBlocksWhenNoTimeAndNoHistory</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>PST-12</t>
+          <t>PST-08</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -2653,17 +2653,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>just above EPS saturates high via D</t>
+          <t>time ok, no history (dt .5, last NaN)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>D4, 2.5/dt=2EPS, lim±100</t>
+          <t>D4, fb2.0, dt.5, fresh</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>+100 (deriv 2097152 exact)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2673,19 +2673,19 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>P-D3 T + saturation</t>
+          <t>P-D3 TF</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>...JustAboveEpsilonSaturatesHigh</t>
+          <t>PIDStructural.DerivativeGuardBlocksWhenTimeOkButNoHistory</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>PST-13</t>
+          <t>PST-09</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2695,17 +2695,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>negative dt robustness</t>
+          <t>fully active (PLUS sign, L47)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>P2/D4, sp1, fb.5, dt−.5</t>
+          <t>D4, seed 2.0/.5, then 2.5/.5</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>1.0 (P-only)</t>
+          <t>+4.0</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2715,34 +2715,34 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>P-D3 invalid input</t>
+          <t>P-D3 TT</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>NegativeDtDisablesDerivativeTerm</t>
+          <t>PIDStructural.DerivativeGuardActiveWhenTimeAndHistory</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>PST-14</t>
+          <t>PST-10</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>resetDerivative</t>
+          <t>updateDerivative</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>history cleared to NaN, guard re-entry</t>
+          <t>history present but dt 0</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>D2, seed 0/.5, reset, then 1.0/.5</t>
+          <t>D4, seed 2.0/.5, then 3.0/dt0</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -2757,39 +2757,39 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>P-D3 TF re-entry</t>
+          <t>P-D3 FT</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>ResetDerivativeClearsHistory</t>
+          <t>PIDStructural.DerivativeGuardBlocksWhenHistoryButNoTime</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>PST-15</t>
+          <t>PST-11</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>updateIntegral</t>
+          <t>updateDerivative</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>windup clamps exactly at limit</t>
+          <t>exact dt==EPS boundary (not &gt;)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>I1/lim.5/out±10, sp1, fb0, dt.5 ×3</t>
+          <t>D4, seed 2.0/.5, then 2.5/dt=EPS</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>0, .5, .5; int .5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2799,39 +2799,39 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>P-D1 T + clamp</t>
+          <t>P-D3 boundary</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>IntegralWindupClampsExactlyAtLimit</t>
+          <t>PIDStructural.DerivativeGuardExactEpsilonIsNotEnoughTime</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>PST-16</t>
+          <t>PST-12</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>output limit</t>
+          <t>updateDerivative</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>exact-boundary passthrough + clamp</t>
+          <t>just above EPS saturates high via D</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>P1/lim±2, sp5, fb 3/2/4</t>
+          <t>D4, 2.5/dt=2EPS, lim±100</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>2.0 / 2.0 / 1.0</t>
+          <t>+100 (deriv 2097152 exact)</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2841,54 +2841,222 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>saturation edges</t>
+          <t>P-D3 T + saturation</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>OutputLimitPassesExactBoundaryThrough</t>
+          <t>PIDStructural.DerivativeGuardJustAboveEpsilonSaturatesHigh</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
+          <t>PST-13</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>updateDerivative</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>negative dt robustness</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>P2/D4, sp1, fb.5, dt−.5</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>1.0 (P-only)</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 invalid input</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.NegativeDtDisablesDerivativeTerm</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>PST-14</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>resetDerivative</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>history cleared to NaN, guard re-entry</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>D2, seed 0/.5, reset, then 1.0/.5</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>P-D3 TF re-entry</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.ResetDerivativeClearsHistory</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>PST-15</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>updateIntegral</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>windup clamps exactly at limit</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>I1/lim.5/out±10, sp1, fb0, dt.5 ×3</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>0, .5, .5; int .5</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>P-D1 T + clamp</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.IntegralWindupClampsExactlyAtLimit</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>PST-16</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>output limit</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>exact-boundary passthrough + clamp</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>P1/lim±2, sp5, fb 3/2/4</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>2.0 / 2.0 / 1.0</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>saturation edges</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.OutputLimitPassesExactBoundaryThrough</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
           <t>PST-17</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>degenerate config</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>zero gains hold zero</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>gains 0, out±5, sp3, fb1</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>0 + int 0</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>degenerate</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>ZeroGainDegenerateConfigHoldsZero</t>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>PIDStructural.ZeroGainDegenerateConfigHoldsZero</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3212,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>c2 independent (only c2 differs vs HST-01)</t>
+          <t>c2 at entry-guard level (req==state → L75 false so L77 masked; strict same-decision flip impossible — see below)</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3320,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>c2 independent</t>
+          <t>c2 at entry-guard level (same masking caveat as H-D5)</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3396,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>BST-07 (mid vs final)</t>
+          <t>BST-07 call1 vs BST-07 call2 (same test, sequential — state flip)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -3547,7 +3715,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>tracks (avg&gt;5)</t>
+          <t>tracks (avg&gt;5, asserted)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -3579,12 +3747,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>(NaN probe, removed — B-D10 demonstrably skips; kept as analyzed behavior, not a workbook row)</t>
+          <t>BST-31</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>c2 (finite)</t>
+          <t>c2 (finite) vs BST-19 — only c2 differs, outcome flips track→hold</t>
         </is>
       </c>
     </row>

</xml_diff>